<commit_message>
:up: ultimo commit antes de tentar arruma os <br> nos flashcards
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards - para criar tabdin.xlsx
+++ b/banco_de_dados/flashcards - para criar tabdin.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\files\programacao\web-design\simulado\banco_de_dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B12E0D5-5498-4915-A696-64D402ABB03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB818E88-E14C-45BB-8A68-09EDF0694CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="8" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1233" uniqueCount="687">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1244" uniqueCount="688">
   <si>
     <t>id</t>
   </si>
@@ -8567,6 +8567,9 @@
   &lt;/li&gt;
 &lt;/ul&gt;</t>
   </si>
+  <si>
+    <t>Rótulos de Linha</t>
+  </si>
 </sst>
 </file>
 
@@ -8601,9 +8604,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="4"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8627,17 +8645,17 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>104776</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>752474</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>180976</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="2" name="assunto">
@@ -8660,7 +8678,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -8670,8 +8688,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="0" y="1285875"/>
-              <a:ext cx="1828800" cy="2524125"/>
+              <a:off x="0" y="1057276"/>
+              <a:ext cx="2581274" cy="2743200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -12229,10 +12247,10 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6F8BECF7-A720-41F1-B6DF-1567D0E7464F}" name="Tabela dinâmica1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="E8:I16" firstHeaderRow="1" firstDataRow="1" firstDataCol="5"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6F8BECF7-A720-41F1-B6DF-1567D0E7464F}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="E8:E67" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="7">
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+    <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
       <items count="279">
         <item x="0"/>
         <item x="4"/>
@@ -12514,13 +12532,8 @@
         <item x="55"/>
         <item x="58"/>
       </items>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
-          <x14:pivotField fillDownLabels="1"/>
-        </ext>
-      </extLst>
     </pivotField>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+    <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
       <items count="11">
         <item x="0"/>
         <item h="1" x="10"/>
@@ -12534,13 +12547,8 @@
         <item h="1" x="2"/>
         <item h="1" x="5"/>
       </items>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
-          <x14:pivotField fillDownLabels="1"/>
-        </ext>
-      </extLst>
     </pivotField>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+    <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
       <items count="43">
         <item h="1" x="18"/>
         <item h="1" x="33"/>
@@ -12559,14 +12567,14 @@
         <item h="1" x="1"/>
         <item h="1" x="20"/>
         <item h="1" x="11"/>
-        <item x="9"/>
+        <item h="1" x="9"/>
         <item h="1" x="2"/>
         <item h="1" x="0"/>
         <item h="1" x="27"/>
         <item h="1" x="3"/>
         <item h="1" x="28"/>
         <item h="1" x="12"/>
-        <item h="1" x="19"/>
+        <item x="19"/>
         <item h="1" x="10"/>
         <item h="1" x="26"/>
         <item h="1" x="14"/>
@@ -12586,13 +12594,8 @@
         <item h="1" x="5"/>
         <item h="1" x="36"/>
       </items>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
-          <x14:pivotField fillDownLabels="1"/>
-        </ext>
-      </extLst>
     </pivotField>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+    <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
       <items count="278">
         <item x="72"/>
         <item x="41"/>
@@ -12873,13 +12876,8 @@
         <item x="157"/>
         <item x="195"/>
       </items>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
-          <x14:pivotField fillDownLabels="1"/>
-        </ext>
-      </extLst>
     </pivotField>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+    <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
       <items count="278">
         <item x="192"/>
         <item x="181"/>
@@ -12993,7 +12991,7 @@
         <item x="199"/>
         <item x="265"/>
         <item x="163"/>
-        <item x="268"/>
+        <item n="&lt;ul&gt;_x000a_  &lt;li&gt;&lt;strong&gt;Principais Indicadores de Tempo&lt;/strong&gt;_x000a_    &lt;ul&gt;_x000a_      &lt;li&gt;&lt;strong&gt;MTBF (Mean Time Between Failures):&lt;/strong&gt; Tempo médio entre falhas. Aplicado a itens &lt;u&gt;reparáveis&lt;/u&gt;. Mede a confiabilidade do processo.&lt;/li&gt;_x000a_      &lt;li&gt;&lt;strong&gt;MTT" x="268"/>
         <item x="200"/>
         <item x="221"/>
         <item x="250"/>
@@ -13160,26 +13158,9 @@
         <item x="56"/>
         <item x="57"/>
       </items>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
-          <x14:pivotField fillDownLabels="1"/>
-        </ext>
-      </extLst>
     </pivotField>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
-          <x14:pivotField fillDownLabels="1"/>
-        </ext>
-      </extLst>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
-          <x14:pivotField fillDownLabels="1"/>
-        </ext>
-      </extLst>
-    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="5">
     <field x="1"/>
@@ -13188,48 +13169,183 @@
     <field x="3"/>
     <field x="4"/>
   </rowFields>
-  <rowItems count="8">
+  <rowItems count="59">
     <i>
       <x/>
-      <x v="17"/>
-      <x v="11"/>
-      <x v="268"/>
-      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="24"/>
     </i>
     <i r="2">
-      <x v="12"/>
-      <x v="151"/>
-      <x v="73"/>
+      <x v="50"/>
+    </i>
+    <i r="3">
+      <x v="80"/>
+    </i>
+    <i r="4">
+      <x v="168"/>
     </i>
     <i r="2">
-      <x v="13"/>
-      <x v="92"/>
-      <x v="19"/>
+      <x v="51"/>
+    </i>
+    <i r="3">
+      <x/>
+    </i>
+    <i r="4">
+      <x v="163"/>
     </i>
     <i r="2">
-      <x v="199"/>
-      <x v="132"/>
-      <x v="112"/>
+      <x v="52"/>
+    </i>
+    <i r="3">
+      <x v="241"/>
+    </i>
+    <i r="4">
+      <x v="188"/>
     </i>
     <i r="2">
-      <x v="200"/>
-      <x v="84"/>
-      <x v="67"/>
+      <x v="53"/>
+    </i>
+    <i r="3">
+      <x v="51"/>
+    </i>
+    <i r="4">
+      <x v="211"/>
     </i>
     <i r="2">
-      <x v="268"/>
-      <x v="62"/>
-      <x v="243"/>
+      <x v="54"/>
+    </i>
+    <i r="3">
+      <x v="96"/>
+    </i>
+    <i r="4">
+      <x v="177"/>
     </i>
     <i r="2">
-      <x v="269"/>
-      <x v="91"/>
-      <x v="17"/>
+      <x v="128"/>
+    </i>
+    <i r="3">
+      <x v="158"/>
+    </i>
+    <i r="4">
+      <x v="125"/>
     </i>
     <i r="2">
-      <x v="270"/>
-      <x v="11"/>
-      <x v="21"/>
+      <x v="129"/>
+    </i>
+    <i r="3">
+      <x v="260"/>
+    </i>
+    <i r="4">
+      <x v="200"/>
+    </i>
+    <i r="2">
+      <x v="144"/>
+    </i>
+    <i r="3">
+      <x v="236"/>
+    </i>
+    <i r="4">
+      <x v="48"/>
+    </i>
+    <i r="2">
+      <x v="151"/>
+    </i>
+    <i r="3">
+      <x v="150"/>
+    </i>
+    <i r="4">
+      <x v="35"/>
+    </i>
+    <i r="2">
+      <x v="213"/>
+    </i>
+    <i r="3">
+      <x v="15"/>
+    </i>
+    <i r="4">
+      <x v="151"/>
+    </i>
+    <i r="2">
+      <x v="214"/>
+    </i>
+    <i r="3">
+      <x v="13"/>
+    </i>
+    <i r="4">
+      <x v="199"/>
+    </i>
+    <i r="2">
+      <x v="215"/>
+    </i>
+    <i r="3">
+      <x v="218"/>
+    </i>
+    <i r="4">
+      <x v="14"/>
+    </i>
+    <i r="2">
+      <x v="216"/>
+    </i>
+    <i r="3">
+      <x v="156"/>
+    </i>
+    <i r="4">
+      <x v="26"/>
+    </i>
+    <i r="2">
+      <x v="217"/>
+    </i>
+    <i r="3">
+      <x v="155"/>
+    </i>
+    <i r="4">
+      <x v="20"/>
+    </i>
+    <i r="2">
+      <x v="218"/>
+    </i>
+    <i r="3">
+      <x v="29"/>
+    </i>
+    <i r="4">
+      <x v="201"/>
+    </i>
+    <i r="2">
+      <x v="219"/>
+    </i>
+    <i r="3">
+      <x v="53"/>
+    </i>
+    <i r="4">
+      <x v="190"/>
+    </i>
+    <i r="2">
+      <x v="220"/>
+    </i>
+    <i r="3">
+      <x v="257"/>
+    </i>
+    <i r="4">
+      <x v="159"/>
+    </i>
+    <i r="2">
+      <x v="254"/>
+    </i>
+    <i r="3">
+      <x v="247"/>
+    </i>
+    <i r="4">
+      <x v="274"/>
+    </i>
+    <i r="2">
+      <x v="255"/>
+    </i>
+    <i r="3">
+      <x v="31"/>
+    </i>
+    <i r="4">
+      <x v="44"/>
     </i>
   </rowItems>
   <colItems count="1">
@@ -13238,7 +13354,7 @@
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" fillDownLabelsDefault="1" hideValuesRow="1"/>
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
     </ext>
     <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
       <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
@@ -13260,14 +13376,14 @@
         <i x="25"/>
         <i x="30"/>
         <i x="11"/>
-        <i x="9" s="1"/>
+        <i x="9"/>
         <i x="2"/>
         <i x="0"/>
         <i x="27"/>
         <i x="3"/>
         <i x="28"/>
         <i x="12"/>
-        <i x="19"/>
+        <i x="19" s="1"/>
         <i x="10"/>
         <i x="13"/>
         <i x="31"/>
@@ -13331,7 +13447,7 @@
 
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="assunto" xr10:uid="{A255312C-2581-4C0E-AEEA-E3503A0C3A02}" cache="SegmentaçãodeDados_assunto" caption="assunto" rowHeight="241300"/>
+  <slicer name="assunto" xr10:uid="{A255312C-2581-4C0E-AEEA-E3503A0C3A02}" cache="SegmentaçãodeDados_assunto" caption="assunto" startItem="6" rowHeight="241300"/>
   <slicer name="disciplina" xr10:uid="{B21AC6A2-0110-4244-808E-21E4413A4585}" cache="SegmentaçãodeDados_disciplina" caption="disciplina" rowHeight="241300"/>
 </slicers>
 </file>
@@ -20095,168 +20211,315 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC24E7D0-197D-4DBF-897D-17C308A658F4}">
-  <dimension ref="E8:I16"/>
+  <dimension ref="E8:E67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="35" customWidth="1"/>
-    <col min="5" max="5" width="31.42578125" customWidth="1"/>
+    <col min="5" max="5" width="255.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="39.85546875" customWidth="1"/>
     <col min="7" max="7" width="7" customWidth="1"/>
     <col min="8" max="8" width="33" customWidth="1"/>
-    <col min="9" max="9" width="114.42578125" customWidth="1"/>
+    <col min="9" max="9" width="255.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="5:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E9" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="9" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F9" t="s">
-        <v>55</v>
-      </c>
-      <c r="G9">
-        <v>24</v>
-      </c>
-      <c r="H9" t="s">
-        <v>56</v>
-      </c>
-      <c r="I9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E10" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" t="s">
-        <v>55</v>
-      </c>
-      <c r="G10">
-        <v>25</v>
-      </c>
-      <c r="H10" t="s">
-        <v>58</v>
-      </c>
-      <c r="I10" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F11" t="s">
-        <v>55</v>
-      </c>
-      <c r="G11">
-        <v>41</v>
-      </c>
-      <c r="H11" t="s">
-        <v>66</v>
-      </c>
-      <c r="I11" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="12" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E12" t="s">
-        <v>7</v>
-      </c>
-      <c r="F12" t="s">
-        <v>55</v>
-      </c>
-      <c r="G12">
-        <v>364</v>
-      </c>
-      <c r="H12" t="s">
-        <v>665</v>
-      </c>
-      <c r="I12" t="s">
-        <v>666</v>
-      </c>
-    </row>
-    <row r="13" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E13" t="s">
-        <v>7</v>
-      </c>
-      <c r="F13" t="s">
-        <v>55</v>
-      </c>
-      <c r="G13">
-        <v>365</v>
-      </c>
-      <c r="H13" t="s">
-        <v>667</v>
-      </c>
-      <c r="I13" t="s">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="14" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E14" t="s">
-        <v>7</v>
-      </c>
-      <c r="F14" t="s">
-        <v>55</v>
-      </c>
-      <c r="G14" t="s">
-        <v>60</v>
-      </c>
-      <c r="H14" t="s">
-        <v>61</v>
-      </c>
-      <c r="I14" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="15" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E15" t="s">
-        <v>7</v>
-      </c>
-      <c r="F15" t="s">
-        <v>55</v>
-      </c>
-      <c r="G15" t="s">
-        <v>63</v>
-      </c>
-      <c r="H15" t="s">
-        <v>64</v>
-      </c>
-      <c r="I15" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="16" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E16" t="s">
-        <v>7</v>
-      </c>
-      <c r="F16" t="s">
-        <v>55</v>
-      </c>
-      <c r="G16" t="s">
-        <v>68</v>
-      </c>
-      <c r="H16" t="s">
-        <v>69</v>
-      </c>
-      <c r="I16" t="s">
-        <v>70</v>
+    </row>
+    <row r="10" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E10" s="3" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="11" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E11" s="4">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E12" s="5" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="13" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E13" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="14" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E14" s="4">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="15" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E15" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="16" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E16" s="6" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E17" s="4">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E18" s="5" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E19" s="6" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E20" s="4">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E21" s="5" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="22" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E22" s="6" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="23" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E23" s="4">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E24" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="25" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E25" s="6" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="26" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E26" s="4">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="27" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E27" s="5" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="28" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E28" s="6" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="29" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E29" s="4">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="30" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E30" s="5" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="31" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E31" s="6" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="32" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E32" s="4">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="33" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E33" s="5" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="34" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E34" s="6" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="35" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E35" s="4">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="36" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E36" s="5" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="37" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E37" s="6" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="38" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E38" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="39" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E39" s="5" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="40" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E40" s="6" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="41" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E41" s="4" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="42" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E42" s="5" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="43" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E43" s="6" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="44" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E44" s="4" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="45" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E45" s="5" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="46" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E46" s="6" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="47" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E47" s="4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="48" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E48" s="5" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="49" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E49" s="6" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="50" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E50" s="4" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="51" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E51" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="52" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E52" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="53" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E53" s="4" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="54" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E54" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="55" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E55" s="6" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="56" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E56" s="4" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="57" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E57" s="5" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="58" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E58" s="6" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="59" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E59" s="4" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="60" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E60" s="5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="61" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E61" s="6" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="62" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E62" s="4" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="63" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E63" s="5" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="64" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E64" s="6" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="65" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E65" s="4" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="66" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E66" s="5" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="67" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E67" s="6" t="s">
+        <v>492</v>
       </c>
     </row>
   </sheetData>

</xml_diff>